<commit_message>
Controle de produção e de serviço: novo estudo, com treinamento e planilha
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="71208899"/>
-        <c:axId val="38846236"/>
+        <c:axId val="667035"/>
+        <c:axId val="13567041"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="71208899"/>
+        <c:axId val="667035"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38846236"/>
+        <c:crossAx val="13567041"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="38846236"/>
+        <c:axId val="13567041"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71208899"/>
+        <c:crossAx val="667035"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="86246838"/>
-        <c:axId val="76412950"/>
+        <c:axId val="83770008"/>
+        <c:axId val="72310626"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86246838"/>
+        <c:axId val="83770008"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76412950"/>
+        <c:crossAx val="72310626"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="76412950"/>
+        <c:axId val="72310626"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86246838"/>
+        <c:crossAx val="83770008"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="25305073"/>
-        <c:axId val="86689033"/>
+        <c:axId val="3006611"/>
+        <c:axId val="16144123"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="25305073"/>
+        <c:axId val="3006611"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86689033"/>
+        <c:crossAx val="16144123"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86689033"/>
+        <c:axId val="16144123"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25305073"/>
+        <c:crossAx val="3006611"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>

</xml_diff>

<commit_message>
Liberação e produto não conforme: novo estudo, com treinamento e planilha
A matriz do estudo da ISO 9001 passa a agrupar, por seção, os estudos que
cobrem três itens ou mais, para o texto caber na célula.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="667035"/>
-        <c:axId val="13567041"/>
+        <c:axId val="59633425"/>
+        <c:axId val="54757049"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="667035"/>
+        <c:axId val="59633425"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13567041"/>
+        <c:crossAx val="54757049"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="13567041"/>
+        <c:axId val="54757049"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="667035"/>
+        <c:crossAx val="59633425"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="83770008"/>
-        <c:axId val="72310626"/>
+        <c:axId val="41469157"/>
+        <c:axId val="92326957"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="83770008"/>
+        <c:axId val="41469157"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72310626"/>
+        <c:crossAx val="92326957"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="72310626"/>
+        <c:axId val="92326957"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83770008"/>
+        <c:crossAx val="41469157"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="3006611"/>
-        <c:axId val="16144123"/>
+        <c:axId val="96913825"/>
+        <c:axId val="92690000"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="3006611"/>
+        <c:axId val="96913825"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16144123"/>
+        <c:crossAx val="92690000"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="16144123"/>
+        <c:axId val="92690000"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3006611"/>
+        <c:crossAx val="96913825"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -7693,16 +7693,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
+    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H26 J7:J26" type="date">
+      <formula1>36526</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Número do requisito, como na aba Diagnóstico" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7:C26" type="list">
       <formula1>"4.1,4.2,4.3,4.4,5.1.1,5.1.2,5.2,5.3,6.1,6.2,6.3,7.1.1,7.1.3,7.1.4,7.1.5,7.1.6,7.2,7.3,7.4,7.5,8.1,8.2.1,8.2.2,8.2.3,8.2.4,8.3,8.4.1,8.4.2,8.4.3,8.5.1,8.5.2,8.5.3,8.5.4,8.5.5,8.5.6,8.6,8.7,9.1.1,9.1.2,9.1.3,9.2,9.3,10.1,10.2,10.3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Não iniciada, Em andamento, Concluída ou Cancelada" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I7:I26" type="list">
       <formula1>"Não iniciada,Em andamento,Concluída,Cancelada"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H26 J7:J26" type="date">
-      <formula1>36526</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Requisitos do cliente e análise de pedidos: novo estudo, com treinamento e planilha
A legenda da matriz do estudo da ISO 9001 passa a dizer o que ainda falta
cobrir na seção 8.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="59633425"/>
-        <c:axId val="54757049"/>
+        <c:axId val="97218562"/>
+        <c:axId val="27801338"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="59633425"/>
+        <c:axId val="97218562"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54757049"/>
+        <c:crossAx val="27801338"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="54757049"/>
+        <c:axId val="27801338"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59633425"/>
+        <c:crossAx val="97218562"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="41469157"/>
-        <c:axId val="92326957"/>
+        <c:axId val="80925580"/>
+        <c:axId val="92711190"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="41469157"/>
+        <c:axId val="80925580"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92326957"/>
+        <c:crossAx val="92711190"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="92326957"/>
+        <c:axId val="92711190"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41469157"/>
+        <c:crossAx val="80925580"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="96913825"/>
-        <c:axId val="92690000"/>
+        <c:axId val="67397486"/>
+        <c:axId val="23364355"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="96913825"/>
+        <c:axId val="67397486"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92690000"/>
+        <c:crossAx val="23364355"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="92690000"/>
+        <c:axId val="23364355"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96913825"/>
+        <c:crossAx val="67397486"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -7693,16 +7693,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H26 J7:J26" type="date">
-      <formula1>36526</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Número do requisito, como na aba Diagnóstico" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7:C26" type="list">
       <formula1>"4.1,4.2,4.3,4.4,5.1.1,5.1.2,5.2,5.3,6.1,6.2,6.3,7.1.1,7.1.3,7.1.4,7.1.5,7.1.6,7.2,7.3,7.4,7.5,8.1,8.2.1,8.2.2,8.2.3,8.2.4,8.3,8.4.1,8.4.2,8.4.3,8.5.1,8.5.2,8.5.3,8.5.4,8.5.5,8.5.6,8.6,8.7,9.1.1,9.1.2,9.1.3,9.2,9.3,10.1,10.2,10.3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Não iniciada, Em andamento, Concluída ou Cancelada" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I7:I26" type="list">
       <formula1>"Não iniciada,Em andamento,Concluída,Cancelada"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H26 J7:J26" type="date">
+      <formula1>36526</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Projeto e desenvolvimento: novo estudo, com treinamento e planilha
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="97218562"/>
-        <c:axId val="27801338"/>
+        <c:axId val="70520543"/>
+        <c:axId val="40335964"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="97218562"/>
+        <c:axId val="70520543"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27801338"/>
+        <c:crossAx val="40335964"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="27801338"/>
+        <c:axId val="40335964"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97218562"/>
+        <c:crossAx val="70520543"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="80925580"/>
-        <c:axId val="92711190"/>
+        <c:axId val="74217605"/>
+        <c:axId val="59576086"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="80925580"/>
+        <c:axId val="74217605"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92711190"/>
+        <c:crossAx val="59576086"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="92711190"/>
+        <c:axId val="59576086"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80925580"/>
+        <c:crossAx val="74217605"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="67397486"/>
-        <c:axId val="23364355"/>
+        <c:axId val="53032538"/>
+        <c:axId val="71788378"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="67397486"/>
+        <c:axId val="53032538"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23364355"/>
+        <c:crossAx val="71788378"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23364355"/>
+        <c:axId val="71788378"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67397486"/>
+        <c:crossAx val="53032538"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>

</xml_diff>

<commit_message>
Escopo e liderança: novo estudo, com treinamento e planilha
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="70520543"/>
-        <c:axId val="40335964"/>
+        <c:axId val="53475626"/>
+        <c:axId val="18090036"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="70520543"/>
+        <c:axId val="53475626"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40335964"/>
+        <c:crossAx val="18090036"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40335964"/>
+        <c:axId val="18090036"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70520543"/>
+        <c:crossAx val="53475626"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="74217605"/>
-        <c:axId val="59576086"/>
+        <c:axId val="97200023"/>
+        <c:axId val="5983360"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="74217605"/>
+        <c:axId val="97200023"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59576086"/>
+        <c:crossAx val="5983360"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59576086"/>
+        <c:axId val="5983360"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74217605"/>
+        <c:crossAx val="97200023"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="53032538"/>
-        <c:axId val="71788378"/>
+        <c:axId val="60174096"/>
+        <c:axId val="95958665"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="53032538"/>
+        <c:axId val="60174096"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71788378"/>
+        <c:crossAx val="95958665"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71788378"/>
+        <c:axId val="95958665"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53032538"/>
+        <c:crossAx val="60174096"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>

</xml_diff>

<commit_message>
Calibração e recursos de medição: novo estudo, com treinamento e planilha
A faixa de apoio da figura do painel passa a ter quatro caixas, e a legenda
da matriz do estudo da ISO 9001 diz o que ainda falta na seção 7.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="53475626"/>
-        <c:axId val="18090036"/>
+        <c:axId val="50239947"/>
+        <c:axId val="37491786"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="53475626"/>
+        <c:axId val="50239947"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18090036"/>
+        <c:crossAx val="37491786"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="18090036"/>
+        <c:axId val="37491786"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53475626"/>
+        <c:crossAx val="50239947"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="97200023"/>
-        <c:axId val="5983360"/>
+        <c:axId val="74200296"/>
+        <c:axId val="53330837"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="97200023"/>
+        <c:axId val="74200296"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5983360"/>
+        <c:crossAx val="53330837"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5983360"/>
+        <c:axId val="53330837"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97200023"/>
+        <c:crossAx val="74200296"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="60174096"/>
-        <c:axId val="95958665"/>
+        <c:axId val="71928617"/>
+        <c:axId val="33413043"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="60174096"/>
+        <c:axId val="71928617"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95958665"/>
+        <c:crossAx val="33413043"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95958665"/>
+        <c:axId val="33413043"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60174096"/>
+        <c:crossAx val="71928617"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -7693,16 +7693,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
+    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H26 J7:J26" type="date">
+      <formula1>36526</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Número do requisito, como na aba Diagnóstico" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7:C26" type="list">
       <formula1>"4.1,4.2,4.3,4.4,5.1.1,5.1.2,5.2,5.3,6.1,6.2,6.3,7.1.1,7.1.3,7.1.4,7.1.5,7.1.6,7.2,7.3,7.4,7.5,8.1,8.2.1,8.2.2,8.2.3,8.2.4,8.3,8.4.1,8.4.2,8.4.3,8.5.1,8.5.2,8.5.3,8.5.4,8.5.5,8.5.6,8.6,8.7,9.1.1,9.1.2,9.1.3,9.2,9.3,10.1,10.2,10.3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Não iniciada, Em andamento, Concluída ou Cancelada" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I7:I26" type="list">
       <formula1>"Não iniciada,Em andamento,Concluída,Cancelada"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H26 J7:J26" type="date">
-      <formula1>36526</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Recursos, infraestrutura e ambiente: novo estudo, com treinamento e planilha
Cobre os requisitos 7.1.1 a 7.1.4: as pessoas dimensionadas pela demanda do
pico, a preventiva e a contingência da infraestrutura, a disponibilidade e os
fatores do ambiente. A faixa de apoio da figura do painel passa a ter cinco
caixas, e a matriz do estudo da ISO 9001 só deixa sem estudo os requisitos
7.1.6 e 8.5.5. O painel também corrige a contagem dos estudos em sequência.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="50239947"/>
-        <c:axId val="37491786"/>
+        <c:axId val="60108320"/>
+        <c:axId val="58669821"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50239947"/>
+        <c:axId val="60108320"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37491786"/>
+        <c:crossAx val="58669821"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="37491786"/>
+        <c:axId val="58669821"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50239947"/>
+        <c:crossAx val="60108320"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="74200296"/>
-        <c:axId val="53330837"/>
+        <c:axId val="89641111"/>
+        <c:axId val="90118626"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="74200296"/>
+        <c:axId val="89641111"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53330837"/>
+        <c:crossAx val="90118626"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="53330837"/>
+        <c:axId val="90118626"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74200296"/>
+        <c:crossAx val="89641111"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="71928617"/>
-        <c:axId val="33413043"/>
+        <c:axId val="19199252"/>
+        <c:axId val="9857682"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="71928617"/>
+        <c:axId val="19199252"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33413043"/>
+        <c:crossAx val="9857682"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="33413043"/>
+        <c:axId val="9857682"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71928617"/>
+        <c:crossAx val="19199252"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -7693,16 +7693,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H26 J7:J26" type="date">
-      <formula1>36526</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Número do requisito, como na aba Diagnóstico" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C7:C26" type="list">
       <formula1>"4.1,4.2,4.3,4.4,5.1.1,5.1.2,5.2,5.3,6.1,6.2,6.3,7.1.1,7.1.3,7.1.4,7.1.5,7.1.6,7.2,7.3,7.4,7.5,8.1,8.2.1,8.2.2,8.2.3,8.2.4,8.3,8.4.1,8.4.2,8.4.3,8.5.1,8.5.2,8.5.3,8.5.4,8.5.5,8.5.6,8.6,8.7,9.1.1,9.1.2,9.1.3,9.2,9.3,10.1,10.2,10.3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Não iniciada, Em andamento, Concluída ou Cancelada" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I7:I26" type="list">
       <formula1>"Não iniciada,Em andamento,Concluída,Cancelada"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H26 J7:J26" type="date">
+      <formula1>36526</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Conhecimento organizacional e pós-entrega: novo estudo, com treinamento e planilha
Cobre os requisitos 7.1.6 e 8.5.5: o mapa do conhecimento com a exposição de
cada um, as lições aprendidas com destino, a política de pós-entrega com os
prazos da lei e do contrato, e os atendimentos com prazo e causa. Com ele,
todos os requisitos da matriz do estudo da ISO 9001 têm estudo. A faixa de
apoio da figura do painel passa a ter seis caixas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="60108320"/>
-        <c:axId val="58669821"/>
+        <c:axId val="24183182"/>
+        <c:axId val="42493779"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="60108320"/>
+        <c:axId val="24183182"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58669821"/>
+        <c:crossAx val="42493779"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58669821"/>
+        <c:axId val="42493779"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60108320"/>
+        <c:crossAx val="24183182"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="89641111"/>
-        <c:axId val="90118626"/>
+        <c:axId val="66956121"/>
+        <c:axId val="91051188"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="89641111"/>
+        <c:axId val="66956121"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90118626"/>
+        <c:crossAx val="91051188"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="90118626"/>
+        <c:axId val="91051188"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89641111"/>
+        <c:crossAx val="66956121"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="19199252"/>
-        <c:axId val="9857682"/>
+        <c:axId val="57648159"/>
+        <c:axId val="87882434"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="19199252"/>
+        <c:axId val="57648159"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9857682"/>
+        <c:crossAx val="87882434"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9857682"/>
+        <c:axId val="87882434"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19199252"/>
+        <c:crossAx val="57648159"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>

</xml_diff>

<commit_message>
Caso integrado: novo estudo, com treinamento e planilha
Segue dois problemas reais dos exemplos, os atrasos da pizzaria e o filme
fino da indústria, de registro em registro pelos estudos da série, e traz o
calendário anual das atividades do sistema e uma ordem de implantação. O
painel ganha o quinto grupo, "Ver o sistema inteiro", e o estudo da ISO 9001
liga o caso aos requisitos 4.4, 9.1.1 e 10.3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="24183182"/>
-        <c:axId val="42493779"/>
+        <c:axId val="94922281"/>
+        <c:axId val="85654604"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="24183182"/>
+        <c:axId val="94922281"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42493779"/>
+        <c:crossAx val="85654604"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42493779"/>
+        <c:axId val="85654604"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24183182"/>
+        <c:crossAx val="94922281"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="66956121"/>
-        <c:axId val="91051188"/>
+        <c:axId val="33142905"/>
+        <c:axId val="6826028"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="66956121"/>
+        <c:axId val="33142905"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91051188"/>
+        <c:crossAx val="6826028"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="91051188"/>
+        <c:axId val="6826028"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66956121"/>
+        <c:crossAx val="33142905"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="57648159"/>
-        <c:axId val="87882434"/>
+        <c:axId val="10042119"/>
+        <c:axId val="17832702"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="57648159"/>
+        <c:axId val="10042119"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87882434"/>
+        <c:crossAx val="17832702"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="87882434"/>
+        <c:axId val="17832702"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57648159"/>
+        <c:crossAx val="10042119"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>

</xml_diff>

<commit_message>
Técnica de auditoria: novo estudo, com treinamento e planilha
Complementa o estudo de Auditoria interna com o trabalho do auditor em campo,
pela ISO 19011: o funil de perguntas, o tamanho e a escolha da amostra, a
força da evidência e a avaliação dos auditores pela auditoria testemunhada.
O quinto grupo do painel passa a se chamar "Ver o sistema inteiro e
certificar", e o estudo da ISO 9001 liga a técnica ao requisito 9.2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="94922281"/>
-        <c:axId val="85654604"/>
+        <c:axId val="911016"/>
+        <c:axId val="94122530"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="94922281"/>
+        <c:axId val="911016"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85654604"/>
+        <c:crossAx val="94122530"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="85654604"/>
+        <c:axId val="94122530"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94922281"/>
+        <c:crossAx val="911016"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="33142905"/>
-        <c:axId val="6826028"/>
+        <c:axId val="8171689"/>
+        <c:axId val="12236983"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="33142905"/>
+        <c:axId val="8171689"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6826028"/>
+        <c:crossAx val="12236983"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6826028"/>
+        <c:axId val="12236983"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33142905"/>
+        <c:crossAx val="8171689"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="10042119"/>
-        <c:axId val="17832702"/>
+        <c:axId val="46685398"/>
+        <c:axId val="89107729"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="10042119"/>
+        <c:axId val="46685398"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17832702"/>
+        <c:crossAx val="89107729"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="17832702"/>
+        <c:axId val="89107729"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10042119"/>
+        <c:crossAx val="46685398"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>

</xml_diff>

<commit_message>
Processo de certificação: novo estudo, com treinamento e planilha
Cobre o caminho até o certificado e a manutenção dele: a prontidão com os
impeditivos de cada fase, a acreditação, as fases 1 e 2, as não
conformidades maiores e menores com os prazos, o ciclo de três anos e a
transição para a ISO 9001:2026, publicada em 16/09/2026. A indústria se
certifica em dezembro de 2027 pela edição de 2015, e a pizzaria em 2028 pela
de 2026. O estudo da ISO 9001 liga a certificação ao requisito 4.3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="911016"/>
-        <c:axId val="94122530"/>
+        <c:axId val="54370930"/>
+        <c:axId val="22799183"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="911016"/>
+        <c:axId val="54370930"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94122530"/>
+        <c:crossAx val="22799183"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94122530"/>
+        <c:axId val="22799183"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="911016"/>
+        <c:crossAx val="54370930"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="8171689"/>
-        <c:axId val="12236983"/>
+        <c:axId val="66195374"/>
+        <c:axId val="61558577"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="8171689"/>
+        <c:axId val="66195374"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12236983"/>
+        <c:crossAx val="61558577"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="12236983"/>
+        <c:axId val="61558577"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8171689"/>
+        <c:crossAx val="66195374"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="46685398"/>
-        <c:axId val="89107729"/>
+        <c:axId val="75254078"/>
+        <c:axId val="7464398"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="46685398"/>
+        <c:axId val="75254078"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89107729"/>
+        <c:crossAx val="7464398"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="89107729"/>
+        <c:axId val="7464398"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46685398"/>
+        <c:crossAx val="75254078"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>

</xml_diff>

<commit_message>
ISO 9001:2026: novo estudo, com treinamento e planilha
As nove mudanças da edição de 2026, o que não mudou, o diagnóstico das
lacunas com prioridade e o plano de transição até 30/09/2029. Exemplos:
a pizzaria a caminho da certificação inicial e a indústria na transição
da 1ª manutenção. Ligado aos requisitos 4.1, 5.1.1, 5.2, 6.1, 6.3 e 7.3
no estudo ISO 9001, e ao painel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="54370930"/>
-        <c:axId val="22799183"/>
+        <c:axId val="12342977"/>
+        <c:axId val="50859421"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="54370930"/>
+        <c:axId val="12342977"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22799183"/>
+        <c:crossAx val="50859421"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22799183"/>
+        <c:axId val="50859421"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54370930"/>
+        <c:crossAx val="12342977"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="66195374"/>
-        <c:axId val="61558577"/>
+        <c:axId val="85068310"/>
+        <c:axId val="58371430"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="66195374"/>
+        <c:axId val="85068310"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61558577"/>
+        <c:crossAx val="58371430"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61558577"/>
+        <c:axId val="58371430"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66195374"/>
+        <c:crossAx val="85068310"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="75254078"/>
-        <c:axId val="7464398"/>
+        <c:axId val="36418632"/>
+        <c:axId val="84376542"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="75254078"/>
+        <c:axId val="36418632"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7464398"/>
+        <c:crossAx val="84376542"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="7464398"/>
+        <c:axId val="84376542"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75254078"/>
+        <c:crossAx val="36418632"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>

</xml_diff>

<commit_message>
Histograma e CEP: novo estudo, com treinamento e planilha
O histograma com a especificação, o gráfico de média e amplitude com
limites calculados da base, quatro regras de sinal e a capacidade com
Cp e Cpk. Exemplos: o peso da bola de massa da pizzaria, em controle
mas não capaz, e a espessura do filme da extrusora 3, em que o gráfico
avisou cinco dias antes da parada de 18/07/2027. Ligado aos requisitos
8.5.1, 9.1.1 e 9.1.3 no estudo ISO 9001, e ao painel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ISO-9001/ISO-9001-modelo.xlsx
+++ b/ISO-9001/ISO-9001-modelo.xlsx
@@ -3212,11 +3212,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="12342977"/>
-        <c:axId val="50859421"/>
+        <c:axId val="389711"/>
+        <c:axId val="38235936"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="12342977"/>
+        <c:axId val="389711"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3248,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50859421"/>
+        <c:crossAx val="38235936"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3256,7 +3256,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="50859421"/>
+        <c:axId val="38235936"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3296,7 +3296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12342977"/>
+        <c:crossAx val="389711"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -3692,11 +3692,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="85068310"/>
-        <c:axId val="58371430"/>
+        <c:axId val="5229127"/>
+        <c:axId val="91819015"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="85068310"/>
+        <c:axId val="5229127"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3728,7 +3728,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58371430"/>
+        <c:crossAx val="91819015"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3736,7 +3736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58371430"/>
+        <c:axId val="91819015"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -3776,7 +3776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85068310"/>
+        <c:crossAx val="5229127"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
@@ -4172,11 +4172,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="36418632"/>
-        <c:axId val="84376542"/>
+        <c:axId val="4927852"/>
+        <c:axId val="37723710"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="36418632"/>
+        <c:axId val="4927852"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4208,7 +4208,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84376542"/>
+        <c:crossAx val="37723710"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4216,7 +4216,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="84376542"/>
+        <c:axId val="37723710"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -4256,7 +4256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36418632"/>
+        <c:crossAx val="4927852"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>

</xml_diff>